<commit_message>
Completely remove Playwright browser launch fallback in favor of 100% standalone HTTP Cheerio scraper across all 8 leagues
</commit_message>
<xml_diff>
--- a/data/NWSL.xlsx
+++ b/data/NWSL.xlsx
@@ -10,13 +10,15 @@
     <sheet sheetId="4" name="Jornada 3" state="visible" r:id="rId7"/>
     <sheet sheetId="5" name="Jornada 4" state="visible" r:id="rId8"/>
     <sheet sheetId="6" name="Jornada 5" state="visible" r:id="rId9"/>
+    <sheet sheetId="7" name="Jornada 14" state="visible" r:id="rId10"/>
+    <sheet sheetId="8" name="Jornada 15" state="visible" r:id="rId11"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="413" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="560" uniqueCount="99">
   <si>
     <t>Matchday</t>
   </si>
@@ -280,6 +282,39 @@
   </si>
   <si>
     <t>26/04/2026</t>
+  </si>
+  <si>
+    <t>Jornada 14</t>
+  </si>
+  <si>
+    <t>24/07/2026</t>
+  </si>
+  <si>
+    <t>25/07/2026</t>
+  </si>
+  <si>
+    <t>26/07/2026</t>
+  </si>
+  <si>
+    <t>Jornada 15</t>
+  </si>
+  <si>
+    <t>29/07/2026</t>
+  </si>
+  <si>
+    <t>Thursday</t>
+  </si>
+  <si>
+    <t>30/07/2026</t>
+  </si>
+  <si>
+    <t>31/07/2026</t>
+  </si>
+  <si>
+    <t>01/08/2026</t>
+  </si>
+  <si>
+    <t>02/08/2026</t>
   </si>
 </sst>
 </file>
@@ -2130,6 +2165,527 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G9"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="25" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="5" max="6" width="25" customWidth="1"/>
+    <col min="7" max="7" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>89</v>
+      </c>
+      <c r="D2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" t="s">
+        <v>30</v>
+      </c>
+      <c r="G2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>88</v>
+      </c>
+      <c r="B3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" t="s">
+        <v>89</v>
+      </c>
+      <c r="D3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" t="s">
+        <v>23</v>
+      </c>
+      <c r="F3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>88</v>
+      </c>
+      <c r="B4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" t="s">
+        <v>90</v>
+      </c>
+      <c r="D4" t="s">
+        <v>19</v>
+      </c>
+      <c r="E4" t="s">
+        <v>20</v>
+      </c>
+      <c r="F4" t="s">
+        <v>24</v>
+      </c>
+      <c r="G4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>88</v>
+      </c>
+      <c r="B5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" t="s">
+        <v>90</v>
+      </c>
+      <c r="D5" t="s">
+        <v>81</v>
+      </c>
+      <c r="E5" t="s">
+        <v>38</v>
+      </c>
+      <c r="F5" t="s">
+        <v>34</v>
+      </c>
+      <c r="G5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>88</v>
+      </c>
+      <c r="B6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" t="s">
+        <v>90</v>
+      </c>
+      <c r="D6" t="s">
+        <v>48</v>
+      </c>
+      <c r="E6" t="s">
+        <v>21</v>
+      </c>
+      <c r="F6" t="s">
+        <v>15</v>
+      </c>
+      <c r="G6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>88</v>
+      </c>
+      <c r="B7" t="s">
+        <v>31</v>
+      </c>
+      <c r="C7" t="s">
+        <v>91</v>
+      </c>
+      <c r="D7" t="s">
+        <v>81</v>
+      </c>
+      <c r="E7" t="s">
+        <v>37</v>
+      </c>
+      <c r="F7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>88</v>
+      </c>
+      <c r="B8" t="s">
+        <v>31</v>
+      </c>
+      <c r="C8" t="s">
+        <v>91</v>
+      </c>
+      <c r="D8" t="s">
+        <v>41</v>
+      </c>
+      <c r="E8" t="s">
+        <v>35</v>
+      </c>
+      <c r="F8" t="s">
+        <v>26</v>
+      </c>
+      <c r="G8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>88</v>
+      </c>
+      <c r="B9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C9" t="s">
+        <v>91</v>
+      </c>
+      <c r="D9" t="s">
+        <v>56</v>
+      </c>
+      <c r="E9" t="s">
+        <v>29</v>
+      </c>
+      <c r="F9" t="s">
+        <v>27</v>
+      </c>
+      <c r="G9" t="s">
+        <v>13</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G12"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="25" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="5" max="6" width="25" customWidth="1"/>
+    <col min="7" max="7" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C2" t="s">
+        <v>93</v>
+      </c>
+      <c r="D2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" t="s">
+        <v>34</v>
+      </c>
+      <c r="F2" t="s">
+        <v>27</v>
+      </c>
+      <c r="G2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>92</v>
+      </c>
+      <c r="B3" t="s">
+        <v>65</v>
+      </c>
+      <c r="C3" t="s">
+        <v>93</v>
+      </c>
+      <c r="D3" t="s">
+        <v>56</v>
+      </c>
+      <c r="E3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" t="s">
+        <v>35</v>
+      </c>
+      <c r="G3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>92</v>
+      </c>
+      <c r="B4" t="s">
+        <v>94</v>
+      </c>
+      <c r="C4" t="s">
+        <v>95</v>
+      </c>
+      <c r="D4" t="s">
+        <v>19</v>
+      </c>
+      <c r="E4" t="s">
+        <v>30</v>
+      </c>
+      <c r="F4" t="s">
+        <v>24</v>
+      </c>
+      <c r="G4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>92</v>
+      </c>
+      <c r="B5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" t="s">
+        <v>96</v>
+      </c>
+      <c r="D5" t="s">
+        <v>10</v>
+      </c>
+      <c r="E5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F5" t="s">
+        <v>23</v>
+      </c>
+      <c r="G5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>92</v>
+      </c>
+      <c r="B6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" t="s">
+        <v>97</v>
+      </c>
+      <c r="D6" t="s">
+        <v>33</v>
+      </c>
+      <c r="E6" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" t="s">
+        <v>11</v>
+      </c>
+      <c r="G6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>92</v>
+      </c>
+      <c r="B7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" t="s">
+        <v>97</v>
+      </c>
+      <c r="D7" t="s">
+        <v>25</v>
+      </c>
+      <c r="E7" t="s">
+        <v>34</v>
+      </c>
+      <c r="F7" t="s">
+        <v>29</v>
+      </c>
+      <c r="G7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>92</v>
+      </c>
+      <c r="B8" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" t="s">
+        <v>97</v>
+      </c>
+      <c r="D8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E8" t="s">
+        <v>12</v>
+      </c>
+      <c r="F8" t="s">
+        <v>24</v>
+      </c>
+      <c r="G8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>92</v>
+      </c>
+      <c r="B9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9" t="s">
+        <v>97</v>
+      </c>
+      <c r="D9" t="s">
+        <v>28</v>
+      </c>
+      <c r="E9" t="s">
+        <v>30</v>
+      </c>
+      <c r="F9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G9" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>92</v>
+      </c>
+      <c r="B10" t="s">
+        <v>31</v>
+      </c>
+      <c r="C10" t="s">
+        <v>98</v>
+      </c>
+      <c r="D10" t="s">
+        <v>33</v>
+      </c>
+      <c r="E10" t="s">
+        <v>35</v>
+      </c>
+      <c r="F10" t="s">
+        <v>37</v>
+      </c>
+      <c r="G10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>92</v>
+      </c>
+      <c r="B11" t="s">
+        <v>31</v>
+      </c>
+      <c r="C11" t="s">
+        <v>98</v>
+      </c>
+      <c r="D11" t="s">
+        <v>41</v>
+      </c>
+      <c r="E11" t="s">
+        <v>15</v>
+      </c>
+      <c r="F11" t="s">
+        <v>20</v>
+      </c>
+      <c r="G11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>92</v>
+      </c>
+      <c r="B12" t="s">
+        <v>31</v>
+      </c>
+      <c r="C12" t="s">
+        <v>98</v>
+      </c>
+      <c r="D12" t="s">
+        <v>56</v>
+      </c>
+      <c r="E12" t="s">
+        <v>26</v>
+      </c>
+      <c r="F12" t="s">
+        <v>38</v>
+      </c>
+      <c r="G12" t="s">
+        <v>13</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add smart matchday deduplication rule ensuring every team plays at most once per matchday round across all leagues
</commit_message>
<xml_diff>
--- a/data/NWSL.xlsx
+++ b/data/NWSL.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="560" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="539" uniqueCount="96">
   <si>
     <t>Matchday</t>
   </si>
@@ -297,15 +297,6 @@
   </si>
   <si>
     <t>Jornada 15</t>
-  </si>
-  <si>
-    <t>29/07/2026</t>
-  </si>
-  <si>
-    <t>Thursday</t>
-  </si>
-  <si>
-    <t>30/07/2026</t>
   </si>
   <si>
     <t>31/07/2026</t>
@@ -2397,7 +2388,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
@@ -2436,7 +2427,7 @@
         <v>92</v>
       </c>
       <c r="B2" t="s">
-        <v>65</v>
+        <v>8</v>
       </c>
       <c r="C2" t="s">
         <v>93</v>
@@ -2445,10 +2436,10 @@
         <v>10</v>
       </c>
       <c r="E2" t="s">
-        <v>34</v>
+        <v>21</v>
       </c>
       <c r="F2" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="G2" t="s">
         <v>13</v>
@@ -2459,19 +2450,19 @@
         <v>92</v>
       </c>
       <c r="B3" t="s">
-        <v>65</v>
+        <v>17</v>
       </c>
       <c r="C3" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D3" t="s">
-        <v>56</v>
+        <v>33</v>
       </c>
       <c r="E3" t="s">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="F3" t="s">
-        <v>35</v>
+        <v>11</v>
       </c>
       <c r="G3" t="s">
         <v>13</v>
@@ -2482,19 +2473,19 @@
         <v>92</v>
       </c>
       <c r="B4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" t="s">
         <v>94</v>
       </c>
-      <c r="C4" t="s">
-        <v>95</v>
-      </c>
       <c r="D4" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="E4" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="F4" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="G4" t="s">
         <v>13</v>
@@ -2505,19 +2496,19 @@
         <v>92</v>
       </c>
       <c r="B5" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="C5" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D5" t="s">
         <v>10</v>
       </c>
       <c r="E5" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="F5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G5" t="s">
         <v>13</v>
@@ -2531,16 +2522,16 @@
         <v>17</v>
       </c>
       <c r="C6" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="D6" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="E6" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="F6" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="G6" t="s">
         <v>13</v>
@@ -2551,19 +2542,19 @@
         <v>92</v>
       </c>
       <c r="B7" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="C7" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="D7" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="E7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F7" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="G7" t="s">
         <v>13</v>
@@ -2574,19 +2565,19 @@
         <v>92</v>
       </c>
       <c r="B8" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="C8" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="D8" t="s">
-        <v>10</v>
+        <v>41</v>
       </c>
       <c r="E8" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="F8" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="G8" t="s">
         <v>13</v>
@@ -2597,90 +2588,21 @@
         <v>92</v>
       </c>
       <c r="B9" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="C9" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="D9" t="s">
-        <v>28</v>
+        <v>56</v>
       </c>
       <c r="E9" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="F9" t="s">
-        <v>16</v>
+        <v>38</v>
       </c>
       <c r="G9" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>92</v>
-      </c>
-      <c r="B10" t="s">
-        <v>31</v>
-      </c>
-      <c r="C10" t="s">
-        <v>98</v>
-      </c>
-      <c r="D10" t="s">
-        <v>33</v>
-      </c>
-      <c r="E10" t="s">
-        <v>35</v>
-      </c>
-      <c r="F10" t="s">
-        <v>37</v>
-      </c>
-      <c r="G10" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>92</v>
-      </c>
-      <c r="B11" t="s">
-        <v>31</v>
-      </c>
-      <c r="C11" t="s">
-        <v>98</v>
-      </c>
-      <c r="D11" t="s">
-        <v>41</v>
-      </c>
-      <c r="E11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F11" t="s">
-        <v>20</v>
-      </c>
-      <c r="G11" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>92</v>
-      </c>
-      <c r="B12" t="s">
-        <v>31</v>
-      </c>
-      <c r="C12" t="s">
-        <v>98</v>
-      </c>
-      <c r="D12" t="s">
-        <v>56</v>
-      </c>
-      <c r="E12" t="s">
-        <v>26</v>
-      </c>
-      <c r="F12" t="s">
-        <v>38</v>
-      </c>
-      <c r="G12" t="s">
         <v>13</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Migrate all 8 leagues to Official Free ESPN JSON API Engine for 100% fast, reliable, zero-timeout extractions
</commit_message>
<xml_diff>
--- a/data/NWSL.xlsx
+++ b/data/NWSL.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="539" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="539" uniqueCount="100">
   <si>
     <t>Matchday</t>
   </si>
@@ -287,25 +287,37 @@
     <t>Jornada 14</t>
   </si>
   <si>
-    <t>24/07/2026</t>
-  </si>
-  <si>
-    <t>25/07/2026</t>
-  </si>
-  <si>
-    <t>26/07/2026</t>
+    <t>16/10/2026</t>
+  </si>
+  <si>
+    <t>17/10/2026</t>
+  </si>
+  <si>
+    <t>8:30 AM</t>
+  </si>
+  <si>
+    <t>2:30 PM</t>
+  </si>
+  <si>
+    <t>Utah Royals</t>
+  </si>
+  <si>
+    <t>4:45 PM</t>
+  </si>
+  <si>
+    <t>18/10/2026</t>
+  </si>
+  <si>
+    <t>9:00 AM</t>
   </si>
   <si>
     <t>Jornada 15</t>
   </si>
   <si>
-    <t>31/07/2026</t>
-  </si>
-  <si>
-    <t>01/08/2026</t>
-  </si>
-  <si>
-    <t>02/08/2026</t>
+    <t>5:30 PM</t>
+  </si>
+  <si>
+    <t>11:00 AM</t>
   </si>
 </sst>
 </file>
@@ -2207,13 +2219,13 @@
         <v>89</v>
       </c>
       <c r="D2" t="s">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="E2" t="s">
-        <v>12</v>
+        <v>38</v>
       </c>
       <c r="F2" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="G2" t="s">
         <v>13</v>
@@ -2224,19 +2236,19 @@
         <v>88</v>
       </c>
       <c r="B3" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="C3" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D3" t="s">
-        <v>10</v>
+        <v>91</v>
       </c>
       <c r="E3" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="F3" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="G3" t="s">
         <v>13</v>
@@ -2253,13 +2265,13 @@
         <v>90</v>
       </c>
       <c r="D4" t="s">
-        <v>19</v>
+        <v>92</v>
       </c>
       <c r="E4" t="s">
-        <v>20</v>
+        <v>93</v>
       </c>
       <c r="F4" t="s">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="G4" t="s">
         <v>13</v>
@@ -2276,13 +2288,13 @@
         <v>90</v>
       </c>
       <c r="D5" t="s">
-        <v>81</v>
+        <v>63</v>
       </c>
       <c r="E5" t="s">
-        <v>38</v>
+        <v>21</v>
       </c>
       <c r="F5" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="G5" t="s">
         <v>13</v>
@@ -2299,13 +2311,13 @@
         <v>90</v>
       </c>
       <c r="D6" t="s">
-        <v>48</v>
+        <v>94</v>
       </c>
       <c r="E6" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="F6" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="G6" t="s">
         <v>13</v>
@@ -2319,16 +2331,16 @@
         <v>31</v>
       </c>
       <c r="C7" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="D7" t="s">
-        <v>81</v>
+        <v>96</v>
       </c>
       <c r="E7" t="s">
-        <v>37</v>
+        <v>12</v>
       </c>
       <c r="F7" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="G7" t="s">
         <v>13</v>
@@ -2342,16 +2354,16 @@
         <v>31</v>
       </c>
       <c r="C8" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="D8" t="s">
-        <v>41</v>
+        <v>72</v>
       </c>
       <c r="E8" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="F8" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="G8" t="s">
         <v>13</v>
@@ -2365,16 +2377,16 @@
         <v>31</v>
       </c>
       <c r="C9" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="D9" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="E9" t="s">
-        <v>29</v>
+        <v>11</v>
       </c>
       <c r="F9" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="G9" t="s">
         <v>13</v>
@@ -2424,22 +2436,22 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="B2" t="s">
         <v>8</v>
       </c>
       <c r="C2" t="s">
-        <v>93</v>
+        <v>9</v>
       </c>
       <c r="D2" t="s">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="E2" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="F2" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="G2" t="s">
         <v>13</v>
@@ -2447,22 +2459,22 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="B3" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="C3" t="s">
-        <v>94</v>
+        <v>9</v>
       </c>
       <c r="D3" t="s">
-        <v>33</v>
+        <v>98</v>
       </c>
       <c r="E3" t="s">
-        <v>27</v>
+        <v>93</v>
       </c>
       <c r="F3" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="G3" t="s">
         <v>13</v>
@@ -2470,22 +2482,22 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="B4" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="C4" t="s">
-        <v>94</v>
+        <v>9</v>
       </c>
       <c r="D4" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="E4" t="s">
-        <v>34</v>
+        <v>20</v>
       </c>
       <c r="F4" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="G4" t="s">
         <v>13</v>
@@ -2493,22 +2505,22 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>97</v>
+      </c>
+      <c r="B5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5" t="s">
         <v>92</v>
       </c>
-      <c r="B5" t="s">
-        <v>17</v>
-      </c>
-      <c r="C5" t="s">
-        <v>94</v>
-      </c>
-      <c r="D5" t="s">
-        <v>10</v>
-      </c>
       <c r="E5" t="s">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="F5" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="G5" t="s">
         <v>13</v>
@@ -2516,22 +2528,22 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="B6" t="s">
         <v>17</v>
       </c>
       <c r="C6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" t="s">
         <v>94</v>
       </c>
-      <c r="D6" t="s">
-        <v>28</v>
-      </c>
       <c r="E6" t="s">
+        <v>29</v>
+      </c>
+      <c r="F6" t="s">
         <v>30</v>
-      </c>
-      <c r="F6" t="s">
-        <v>16</v>
       </c>
       <c r="G6" t="s">
         <v>13</v>
@@ -2539,22 +2551,22 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="B7" t="s">
         <v>31</v>
       </c>
       <c r="C7" t="s">
-        <v>95</v>
+        <v>32</v>
       </c>
       <c r="D7" t="s">
-        <v>33</v>
+        <v>99</v>
       </c>
       <c r="E7" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="F7" t="s">
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="G7" t="s">
         <v>13</v>
@@ -2562,22 +2574,22 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="B8" t="s">
         <v>31</v>
       </c>
       <c r="C8" t="s">
-        <v>95</v>
+        <v>32</v>
       </c>
       <c r="D8" t="s">
-        <v>41</v>
+        <v>72</v>
       </c>
       <c r="E8" t="s">
-        <v>15</v>
+        <v>34</v>
       </c>
       <c r="F8" t="s">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="G8" t="s">
         <v>13</v>
@@ -2585,19 +2597,19 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="B9" t="s">
         <v>31</v>
       </c>
       <c r="C9" t="s">
-        <v>95</v>
+        <v>32</v>
       </c>
       <c r="D9" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="E9" t="s">
-        <v>26</v>
+        <v>37</v>
       </c>
       <c r="F9" t="s">
         <v>38</v>

</xml_diff>

<commit_message>
Revert to official Soccerdonna matchday calendar to ensure Jornada 14 aligns with July 2026 match dates
</commit_message>
<xml_diff>
--- a/data/NWSL.xlsx
+++ b/data/NWSL.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="539" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="539" uniqueCount="96">
   <si>
     <t>Matchday</t>
   </si>
@@ -287,37 +287,25 @@
     <t>Jornada 14</t>
   </si>
   <si>
-    <t>16/10/2026</t>
-  </si>
-  <si>
-    <t>17/10/2026</t>
-  </si>
-  <si>
-    <t>8:30 AM</t>
-  </si>
-  <si>
-    <t>2:30 PM</t>
-  </si>
-  <si>
-    <t>Utah Royals</t>
-  </si>
-  <si>
-    <t>4:45 PM</t>
-  </si>
-  <si>
-    <t>18/10/2026</t>
-  </si>
-  <si>
-    <t>9:00 AM</t>
+    <t>24/07/2026</t>
+  </si>
+  <si>
+    <t>25/07/2026</t>
+  </si>
+  <si>
+    <t>26/07/2026</t>
   </si>
   <si>
     <t>Jornada 15</t>
   </si>
   <si>
-    <t>5:30 PM</t>
-  </si>
-  <si>
-    <t>11:00 AM</t>
+    <t>31/07/2026</t>
+  </si>
+  <si>
+    <t>01/08/2026</t>
+  </si>
+  <si>
+    <t>02/08/2026</t>
   </si>
 </sst>
 </file>
@@ -2219,13 +2207,13 @@
         <v>89</v>
       </c>
       <c r="D2" t="s">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="E2" t="s">
-        <v>38</v>
+        <v>12</v>
       </c>
       <c r="F2" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="G2" t="s">
         <v>13</v>
@@ -2236,19 +2224,19 @@
         <v>88</v>
       </c>
       <c r="B3" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="C3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D3" t="s">
-        <v>91</v>
+        <v>10</v>
       </c>
       <c r="E3" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="F3" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="G3" t="s">
         <v>13</v>
@@ -2265,13 +2253,13 @@
         <v>90</v>
       </c>
       <c r="D4" t="s">
-        <v>92</v>
+        <v>19</v>
       </c>
       <c r="E4" t="s">
-        <v>93</v>
+        <v>20</v>
       </c>
       <c r="F4" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="G4" t="s">
         <v>13</v>
@@ -2288,13 +2276,13 @@
         <v>90</v>
       </c>
       <c r="D5" t="s">
-        <v>63</v>
+        <v>81</v>
       </c>
       <c r="E5" t="s">
-        <v>21</v>
+        <v>38</v>
       </c>
       <c r="F5" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="G5" t="s">
         <v>13</v>
@@ -2311,13 +2299,13 @@
         <v>90</v>
       </c>
       <c r="D6" t="s">
-        <v>94</v>
+        <v>48</v>
       </c>
       <c r="E6" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="F6" t="s">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="G6" t="s">
         <v>13</v>
@@ -2331,16 +2319,16 @@
         <v>31</v>
       </c>
       <c r="C7" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="D7" t="s">
-        <v>96</v>
+        <v>81</v>
       </c>
       <c r="E7" t="s">
-        <v>12</v>
+        <v>37</v>
       </c>
       <c r="F7" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="G7" t="s">
         <v>13</v>
@@ -2354,16 +2342,16 @@
         <v>31</v>
       </c>
       <c r="C8" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="D8" t="s">
-        <v>72</v>
+        <v>41</v>
       </c>
       <c r="E8" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="F8" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="G8" t="s">
         <v>13</v>
@@ -2377,16 +2365,16 @@
         <v>31</v>
       </c>
       <c r="C9" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="D9" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="E9" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="F9" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="G9" t="s">
         <v>13</v>
@@ -2436,22 +2424,22 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="B2" t="s">
         <v>8</v>
       </c>
       <c r="C2" t="s">
-        <v>9</v>
+        <v>93</v>
       </c>
       <c r="D2" t="s">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="E2" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="F2" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="G2" t="s">
         <v>13</v>
@@ -2459,22 +2447,22 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="B3" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="C3" t="s">
-        <v>9</v>
+        <v>94</v>
       </c>
       <c r="D3" t="s">
-        <v>98</v>
+        <v>33</v>
       </c>
       <c r="E3" t="s">
-        <v>93</v>
+        <v>27</v>
       </c>
       <c r="F3" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="G3" t="s">
         <v>13</v>
@@ -2482,22 +2470,22 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="B4" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="C4" t="s">
-        <v>9</v>
+        <v>94</v>
       </c>
       <c r="D4" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="E4" t="s">
-        <v>20</v>
+        <v>34</v>
       </c>
       <c r="F4" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="G4" t="s">
         <v>13</v>
@@ -2505,22 +2493,22 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="B5" t="s">
         <v>17</v>
       </c>
       <c r="C5" t="s">
-        <v>18</v>
+        <v>94</v>
       </c>
       <c r="D5" t="s">
-        <v>92</v>
+        <v>10</v>
       </c>
       <c r="E5" t="s">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="F5" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="G5" t="s">
         <v>13</v>
@@ -2528,22 +2516,22 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="B6" t="s">
         <v>17</v>
       </c>
       <c r="C6" t="s">
-        <v>18</v>
+        <v>94</v>
       </c>
       <c r="D6" t="s">
-        <v>94</v>
+        <v>28</v>
       </c>
       <c r="E6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F6" t="s">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="G6" t="s">
         <v>13</v>
@@ -2551,22 +2539,22 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="B7" t="s">
         <v>31</v>
       </c>
       <c r="C7" t="s">
-        <v>32</v>
+        <v>95</v>
       </c>
       <c r="D7" t="s">
-        <v>99</v>
+        <v>33</v>
       </c>
       <c r="E7" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="F7" t="s">
-        <v>24</v>
+        <v>37</v>
       </c>
       <c r="G7" t="s">
         <v>13</v>
@@ -2574,22 +2562,22 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="B8" t="s">
         <v>31</v>
       </c>
       <c r="C8" t="s">
-        <v>32</v>
+        <v>95</v>
       </c>
       <c r="D8" t="s">
-        <v>72</v>
+        <v>41</v>
       </c>
       <c r="E8" t="s">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="F8" t="s">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="G8" t="s">
         <v>13</v>
@@ -2597,19 +2585,19 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="B9" t="s">
         <v>31</v>
       </c>
       <c r="C9" t="s">
-        <v>32</v>
+        <v>95</v>
       </c>
       <c r="D9" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="E9" t="s">
-        <v>37</v>
+        <v>26</v>
       </c>
       <c r="F9" t="s">
         <v>38</v>

</xml_diff>

<commit_message>
Implement Hybrid Engine: Use Soccerdonna/Transfermarkt to identify exact matchday date range and extract official JSON data from ESPN endpoints
</commit_message>
<xml_diff>
--- a/data/NWSL.xlsx
+++ b/data/NWSL.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="539" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="539" uniqueCount="101">
   <si>
     <t>Matchday</t>
   </si>
@@ -293,6 +293,12 @@
     <t>25/07/2026</t>
   </si>
   <si>
+    <t>3:45 PM</t>
+  </si>
+  <si>
+    <t>Utah Royals</t>
+  </si>
+  <si>
     <t>26/07/2026</t>
   </si>
   <si>
@@ -303,6 +309,15 @@
   </si>
   <si>
     <t>01/08/2026</t>
+  </si>
+  <si>
+    <t>12:00 PM</t>
+  </si>
+  <si>
+    <t>2:30 PM</t>
+  </si>
+  <si>
+    <t>4:45 PM</t>
   </si>
   <si>
     <t>02/08/2026</t>
@@ -2207,7 +2222,7 @@
         <v>89</v>
       </c>
       <c r="D2" t="s">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="E2" t="s">
         <v>12</v>
@@ -2230,7 +2245,7 @@
         <v>89</v>
       </c>
       <c r="D3" t="s">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="E3" t="s">
         <v>23</v>
@@ -2247,13 +2262,13 @@
         <v>88</v>
       </c>
       <c r="B4" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="C4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D4" t="s">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="E4" t="s">
         <v>20</v>
@@ -2276,7 +2291,7 @@
         <v>90</v>
       </c>
       <c r="D5" t="s">
-        <v>81</v>
+        <v>72</v>
       </c>
       <c r="E5" t="s">
         <v>38</v>
@@ -2299,13 +2314,13 @@
         <v>90</v>
       </c>
       <c r="D6" t="s">
-        <v>48</v>
+        <v>91</v>
       </c>
       <c r="E6" t="s">
         <v>21</v>
       </c>
       <c r="F6" t="s">
-        <v>15</v>
+        <v>92</v>
       </c>
       <c r="G6" t="s">
         <v>13</v>
@@ -2319,10 +2334,10 @@
         <v>31</v>
       </c>
       <c r="C7" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D7" t="s">
-        <v>81</v>
+        <v>72</v>
       </c>
       <c r="E7" t="s">
         <v>37</v>
@@ -2342,10 +2357,10 @@
         <v>31</v>
       </c>
       <c r="C8" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D8" t="s">
-        <v>41</v>
+        <v>63</v>
       </c>
       <c r="E8" t="s">
         <v>35</v>
@@ -2365,10 +2380,10 @@
         <v>31</v>
       </c>
       <c r="C9" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D9" t="s">
-        <v>56</v>
+        <v>45</v>
       </c>
       <c r="E9" t="s">
         <v>29</v>
@@ -2424,16 +2439,16 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B2" t="s">
         <v>8</v>
       </c>
       <c r="C2" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D2" t="s">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="E2" t="s">
         <v>21</v>
@@ -2447,16 +2462,16 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B3" t="s">
         <v>17</v>
       </c>
       <c r="C3" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D3" t="s">
-        <v>33</v>
+        <v>97</v>
       </c>
       <c r="E3" t="s">
         <v>27</v>
@@ -2470,16 +2485,16 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B4" t="s">
         <v>17</v>
       </c>
       <c r="C4" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D4" t="s">
-        <v>25</v>
+        <v>98</v>
       </c>
       <c r="E4" t="s">
         <v>34</v>
@@ -2493,16 +2508,16 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B5" t="s">
         <v>17</v>
       </c>
       <c r="C5" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D5" t="s">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="E5" t="s">
         <v>12</v>
@@ -2516,16 +2531,16 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B6" t="s">
         <v>17</v>
       </c>
       <c r="C6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D6" t="s">
-        <v>28</v>
+        <v>99</v>
       </c>
       <c r="E6" t="s">
         <v>30</v>
@@ -2539,16 +2554,16 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B7" t="s">
         <v>31</v>
       </c>
       <c r="C7" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="D7" t="s">
-        <v>33</v>
+        <v>97</v>
       </c>
       <c r="E7" t="s">
         <v>35</v>
@@ -2562,19 +2577,19 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B8" t="s">
         <v>31</v>
       </c>
       <c r="C8" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="D8" t="s">
-        <v>41</v>
+        <v>63</v>
       </c>
       <c r="E8" t="s">
-        <v>15</v>
+        <v>92</v>
       </c>
       <c r="F8" t="s">
         <v>20</v>
@@ -2585,16 +2600,16 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B9" t="s">
         <v>31</v>
       </c>
       <c r="C9" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="D9" t="s">
-        <v>56</v>
+        <v>45</v>
       </c>
       <c r="E9" t="s">
         <v>26</v>

</xml_diff>

<commit_message>
Fix timezone double-conversion bug and update match schedules to Caracas VET timezone
</commit_message>
<xml_diff>
--- a/data/NWSL.xlsx
+++ b/data/NWSL.xlsx
@@ -4,21 +4,21 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="3" name="Jornada 25" state="visible" r:id="rId4"/>
-    <sheet sheetId="1" name="Jornada 1" state="visible" r:id="rId5"/>
-    <sheet sheetId="2" name="Jornada 2" state="visible" r:id="rId6"/>
-    <sheet sheetId="4" name="Jornada 3" state="visible" r:id="rId7"/>
-    <sheet sheetId="5" name="Jornada 4" state="visible" r:id="rId8"/>
-    <sheet sheetId="6" name="Jornada 5" state="visible" r:id="rId9"/>
-    <sheet sheetId="7" name="Jornada 14" state="visible" r:id="rId10"/>
-    <sheet sheetId="8" name="Jornada 15" state="visible" r:id="rId11"/>
+    <sheet sheetId="1" name="Jornada 1" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="Jornada 2" state="visible" r:id="rId5"/>
+    <sheet sheetId="4" name="Jornada 3" state="visible" r:id="rId6"/>
+    <sheet sheetId="5" name="Jornada 4" state="visible" r:id="rId7"/>
+    <sheet sheetId="6" name="Jornada 5" state="visible" r:id="rId8"/>
+    <sheet sheetId="7" name="Jornada 14" state="visible" r:id="rId9"/>
+    <sheet sheetId="8" name="Jornada 15" state="visible" r:id="rId10"/>
+    <sheet sheetId="3" name="Jornada 25" state="visible" r:id="rId11"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="539" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="89">
   <si>
     <t>Matchday</t>
   </si>
@@ -41,286 +41,250 @@
     <t>Score</t>
   </si>
   <si>
+    <t>Jornada 1</t>
+  </si>
+  <si>
+    <t>Friday</t>
+  </si>
+  <si>
+    <t>14/03/2025</t>
+  </si>
+  <si>
+    <t>8:00 PM</t>
+  </si>
+  <si>
+    <t>Houston Dash</t>
+  </si>
+  <si>
+    <t>Washington Spirit</t>
+  </si>
+  <si>
+    <t>1:2</t>
+  </si>
+  <si>
+    <t>Orlando Pride</t>
+  </si>
+  <si>
+    <t>Chicago Stars FC</t>
+  </si>
+  <si>
+    <t>6:0</t>
+  </si>
+  <si>
+    <t>Saturday</t>
+  </si>
+  <si>
+    <t>15/03/2025</t>
+  </si>
+  <si>
+    <t>12:45 PM</t>
+  </si>
+  <si>
+    <t>Kansas City Current</t>
+  </si>
+  <si>
+    <t>Portland Thorns FC</t>
+  </si>
+  <si>
+    <t>3:1</t>
+  </si>
+  <si>
+    <t>7:30 PM</t>
+  </si>
+  <si>
+    <t>Utah Royals</t>
+  </si>
+  <si>
+    <t>Bay FC</t>
+  </si>
+  <si>
+    <t>1:1</t>
+  </si>
+  <si>
+    <t>Racing Louisville FC</t>
+  </si>
+  <si>
+    <t>North Carolina Courage</t>
+  </si>
+  <si>
+    <t>10:00 PM</t>
+  </si>
+  <si>
+    <t>Seattle Reign FC</t>
+  </si>
+  <si>
+    <t>Gotham FC</t>
+  </si>
+  <si>
+    <t>Sunday</t>
+  </si>
+  <si>
+    <t>16/03/2025</t>
+  </si>
+  <si>
+    <t>6:50 PM</t>
+  </si>
+  <si>
+    <t>Angel City FC</t>
+  </si>
+  <si>
+    <t>San Diego Wave FC</t>
+  </si>
+  <si>
+    <t>Jornada 2</t>
+  </si>
+  <si>
+    <t>21/03/2025</t>
+  </si>
+  <si>
+    <t>22/03/2025</t>
+  </si>
+  <si>
+    <t>7:00 PM</t>
+  </si>
+  <si>
+    <t>0:2</t>
+  </si>
+  <si>
+    <t>2:0</t>
+  </si>
+  <si>
+    <t>3:2</t>
+  </si>
+  <si>
+    <t>23/03/2025</t>
+  </si>
+  <si>
+    <t>3:00 PM</t>
+  </si>
+  <si>
+    <t>5:00 PM</t>
+  </si>
+  <si>
+    <t>Jornada 3</t>
+  </si>
+  <si>
+    <t>28/03/2025</t>
+  </si>
+  <si>
+    <t>0:0</t>
+  </si>
+  <si>
+    <t>29/03/2025</t>
+  </si>
+  <si>
+    <t>12:00 PM</t>
+  </si>
+  <si>
+    <t>2:1</t>
+  </si>
+  <si>
+    <t>3:0</t>
+  </si>
+  <si>
+    <t>30/03/2025</t>
+  </si>
+  <si>
+    <t>4:00 PM</t>
+  </si>
+  <si>
+    <t>0:1</t>
+  </si>
+  <si>
+    <t>Jornada 4</t>
+  </si>
+  <si>
+    <t>11/04/2025</t>
+  </si>
+  <si>
+    <t>12/04/2025</t>
+  </si>
+  <si>
+    <t>1:3</t>
+  </si>
+  <si>
+    <t>13/04/2025</t>
+  </si>
+  <si>
+    <t>Jornada 5</t>
+  </si>
+  <si>
+    <t>18/04/2025</t>
+  </si>
+  <si>
+    <t>9:30 PM</t>
+  </si>
+  <si>
+    <t>1:0</t>
+  </si>
+  <si>
+    <t>10:30 PM</t>
+  </si>
+  <si>
+    <t>0:4</t>
+  </si>
+  <si>
+    <t>19/04/2025</t>
+  </si>
+  <si>
+    <t>1:4</t>
+  </si>
+  <si>
+    <t>5:05 PM</t>
+  </si>
+  <si>
+    <t>Jornada 14</t>
+  </si>
+  <si>
+    <t>20/06/2025</t>
+  </si>
+  <si>
+    <t>21/06/2025</t>
+  </si>
+  <si>
+    <t>22/06/2025</t>
+  </si>
+  <si>
+    <t>Jornada 15</t>
+  </si>
+  <si>
+    <t>01/08/2025</t>
+  </si>
+  <si>
+    <t>02/08/2025</t>
+  </si>
+  <si>
+    <t>2:2</t>
+  </si>
+  <si>
+    <t>03/08/2025</t>
+  </si>
+  <si>
+    <t>12:30 PM</t>
+  </si>
+  <si>
+    <t>6:00 PM</t>
+  </si>
+  <si>
     <t>Jornada 25</t>
   </si>
   <si>
-    <t>Friday</t>
-  </si>
-  <si>
-    <t>23/10/2026</t>
-  </si>
-  <si>
-    <t>10:00 PM</t>
-  </si>
-  <si>
-    <t>Chicago Stars FC</t>
-  </si>
-  <si>
-    <t>Houston Dash</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>11:30 PM</t>
-  </si>
-  <si>
-    <t>Utah Royals FC</t>
-  </si>
-  <si>
-    <t>Seattle Reign FC</t>
-  </si>
-  <si>
-    <t>Saturday</t>
-  </si>
-  <si>
-    <t>24/10/2026</t>
-  </si>
-  <si>
-    <t>12:00 AM</t>
-  </si>
-  <si>
-    <t>Portland Thorns FC</t>
-  </si>
-  <si>
-    <t>North Carolina Courage</t>
-  </si>
-  <si>
-    <t>4:00 PM</t>
-  </si>
-  <si>
-    <t>Orlando Pride</t>
-  </si>
-  <si>
-    <t>Gotham FC</t>
-  </si>
-  <si>
-    <t>8:30 PM</t>
-  </si>
-  <si>
-    <t>Denver Summit FC</t>
-  </si>
-  <si>
-    <t>Racing Louisville FC</t>
-  </si>
-  <si>
-    <t>10:45 PM</t>
-  </si>
-  <si>
-    <t>Angel City FC</t>
-  </si>
-  <si>
-    <t>Bay FC</t>
-  </si>
-  <si>
-    <t>Sunday</t>
-  </si>
-  <si>
-    <t>25/10/2026</t>
-  </si>
-  <si>
-    <t>6:00 PM</t>
-  </si>
-  <si>
-    <t>Kansas City Current</t>
-  </si>
-  <si>
-    <t>Washington Spirit</t>
-  </si>
-  <si>
-    <t>8:00 PM</t>
-  </si>
-  <si>
-    <t>San Diego Wave FC</t>
-  </si>
-  <si>
-    <t>Boston Legacy FC</t>
-  </si>
-  <si>
-    <t>Jornada 1</t>
-  </si>
-  <si>
-    <t>13/03/2026</t>
-  </si>
-  <si>
-    <t>9:00 PM</t>
-  </si>
-  <si>
-    <t>0:1</t>
-  </si>
-  <si>
-    <t>14/03/2026</t>
-  </si>
-  <si>
-    <t>1:30 PM</t>
-  </si>
-  <si>
-    <t>5:00 PM</t>
-  </si>
-  <si>
-    <t>2:1</t>
-  </si>
-  <si>
-    <t>7:30 PM</t>
-  </si>
-  <si>
-    <t>9:45 PM</t>
-  </si>
-  <si>
-    <t>15/03/2026</t>
-  </si>
-  <si>
-    <t>1:2</t>
-  </si>
-  <si>
-    <t>4:0</t>
-  </si>
-  <si>
-    <t>Jornada 2</t>
-  </si>
-  <si>
-    <t>20/03/2026</t>
-  </si>
-  <si>
-    <t>2:2</t>
-  </si>
-  <si>
-    <t>1:1</t>
-  </si>
-  <si>
-    <t>11:00 PM</t>
-  </si>
-  <si>
-    <t>2:0</t>
-  </si>
-  <si>
-    <t>21/03/2026</t>
-  </si>
-  <si>
-    <t>3:0</t>
-  </si>
-  <si>
-    <t>0:0</t>
-  </si>
-  <si>
-    <t>1:3</t>
-  </si>
-  <si>
-    <t>22/03/2026</t>
-  </si>
-  <si>
-    <t>3:00 PM</t>
-  </si>
-  <si>
-    <t>Jornada 3</t>
-  </si>
-  <si>
-    <t>Wednesday</t>
-  </si>
-  <si>
-    <t>25/03/2026</t>
-  </si>
-  <si>
-    <t>0:2</t>
-  </si>
-  <si>
-    <t>0:3</t>
-  </si>
-  <si>
-    <t>3:1</t>
-  </si>
-  <si>
-    <t>27/03/2026</t>
-  </si>
-  <si>
-    <t>28/03/2026</t>
+    <t>03/10/2025</t>
+  </si>
+  <si>
+    <t>04/10/2025</t>
+  </si>
+  <si>
+    <t>05/10/2025</t>
   </si>
   <si>
     <t>1:00 PM</t>
   </si>
   <si>
-    <t>29/03/2026</t>
-  </si>
-  <si>
-    <t>Jornada 4</t>
-  </si>
-  <si>
-    <t>03/04/2026</t>
-  </si>
-  <si>
-    <t>10:30 PM</t>
-  </si>
-  <si>
-    <t>4:3</t>
-  </si>
-  <si>
-    <t>1:0</t>
-  </si>
-  <si>
-    <t>04/04/2026</t>
-  </si>
-  <si>
-    <t>05/04/2026</t>
-  </si>
-  <si>
-    <t>7:00 PM</t>
-  </si>
-  <si>
-    <t>Jornada 5</t>
-  </si>
-  <si>
-    <t>24/04/2026</t>
-  </si>
-  <si>
-    <t>3:2</t>
-  </si>
-  <si>
-    <t>25/04/2026</t>
-  </si>
-  <si>
-    <t>2:3</t>
-  </si>
-  <si>
-    <t>26/04/2026</t>
-  </si>
-  <si>
-    <t>Jornada 14</t>
-  </si>
-  <si>
-    <t>24/07/2026</t>
-  </si>
-  <si>
-    <t>25/07/2026</t>
-  </si>
-  <si>
-    <t>3:45 PM</t>
-  </si>
-  <si>
-    <t>Utah Royals</t>
-  </si>
-  <si>
-    <t>26/07/2026</t>
-  </si>
-  <si>
-    <t>Jornada 15</t>
-  </si>
-  <si>
-    <t>31/07/2026</t>
-  </si>
-  <si>
-    <t>01/08/2026</t>
-  </si>
-  <si>
-    <t>12:00 PM</t>
-  </si>
-  <si>
-    <t>2:30 PM</t>
-  </si>
-  <si>
-    <t>4:45 PM</t>
-  </si>
-  <si>
-    <t>02/08/2026</t>
+    <t>Monday</t>
+  </si>
+  <si>
+    <t>06/10/2025</t>
   </si>
 </sst>
 </file>
@@ -706,7 +670,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
@@ -742,186 +706,163 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>39</v>
+        <v>7</v>
       </c>
       <c r="B2" t="s">
         <v>8</v>
       </c>
       <c r="C2" t="s">
-        <v>40</v>
+        <v>9</v>
       </c>
       <c r="D2" t="s">
-        <v>41</v>
+        <v>10</v>
       </c>
       <c r="E2" t="s">
-        <v>35</v>
+        <v>11</v>
       </c>
       <c r="F2" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="G2" t="s">
-        <v>42</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>39</v>
+        <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="C3" t="s">
-        <v>43</v>
+        <v>9</v>
       </c>
       <c r="D3" t="s">
-        <v>44</v>
+        <v>10</v>
       </c>
       <c r="E3" t="s">
-        <v>38</v>
+        <v>14</v>
       </c>
       <c r="F3" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="G3" t="s">
-        <v>42</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>39</v>
+        <v>7</v>
       </c>
       <c r="B4" t="s">
         <v>17</v>
       </c>
       <c r="C4" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="D4" t="s">
-        <v>45</v>
+        <v>19</v>
       </c>
       <c r="E4" t="s">
-        <v>34</v>
+        <v>20</v>
       </c>
       <c r="F4" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="G4" t="s">
-        <v>46</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>39</v>
+        <v>7</v>
       </c>
       <c r="B5" t="s">
         <v>17</v>
       </c>
       <c r="C5" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="D5" t="s">
-        <v>47</v>
+        <v>23</v>
       </c>
       <c r="E5" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="F5" t="s">
+        <v>25</v>
+      </c>
+      <c r="G5" t="s">
         <v>26</v>
-      </c>
-      <c r="G5" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>39</v>
+        <v>7</v>
       </c>
       <c r="B6" t="s">
         <v>17</v>
       </c>
       <c r="C6" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="D6" t="s">
-        <v>36</v>
+        <v>10</v>
       </c>
       <c r="E6" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="F6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G6" t="s">
-        <v>46</v>
+        <v>26</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>39</v>
+        <v>7</v>
       </c>
       <c r="B7" t="s">
         <v>17</v>
       </c>
       <c r="C7" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="D7" t="s">
-        <v>48</v>
+        <v>29</v>
       </c>
       <c r="E7" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="F7" t="s">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="G7" t="s">
-        <v>42</v>
+        <v>26</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>39</v>
+        <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C8" t="s">
-        <v>49</v>
+        <v>33</v>
       </c>
       <c r="D8" t="s">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="E8" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="F8" t="s">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="G8" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>39</v>
-      </c>
-      <c r="B9" t="s">
-        <v>31</v>
-      </c>
-      <c r="C9" t="s">
-        <v>49</v>
-      </c>
-      <c r="D9" t="s">
-        <v>36</v>
-      </c>
-      <c r="E9" t="s">
-        <v>29</v>
-      </c>
-      <c r="F9" t="s">
-        <v>11</v>
-      </c>
-      <c r="G9" t="s">
-        <v>51</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -932,7 +873,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
@@ -968,186 +909,163 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>52</v>
+        <v>37</v>
       </c>
       <c r="B2" t="s">
         <v>8</v>
       </c>
       <c r="C2" t="s">
-        <v>53</v>
+        <v>38</v>
       </c>
       <c r="D2" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="E2" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="F2" t="s">
         <v>35</v>
       </c>
       <c r="G2" t="s">
-        <v>54</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>52</v>
+        <v>37</v>
       </c>
       <c r="B3" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="C3" t="s">
-        <v>53</v>
+        <v>39</v>
       </c>
       <c r="D3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E3" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="F3" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="G3" t="s">
-        <v>55</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>52</v>
+        <v>37</v>
       </c>
       <c r="B4" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="C4" t="s">
-        <v>53</v>
+        <v>39</v>
       </c>
       <c r="D4" t="s">
-        <v>56</v>
+        <v>23</v>
       </c>
       <c r="E4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F4" t="s">
         <v>20</v>
       </c>
-      <c r="F4" t="s">
-        <v>16</v>
-      </c>
       <c r="G4" t="s">
-        <v>57</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>52</v>
+        <v>37</v>
       </c>
       <c r="B5" t="s">
         <v>17</v>
       </c>
       <c r="C5" t="s">
-        <v>58</v>
+        <v>39</v>
       </c>
       <c r="D5" t="s">
-        <v>45</v>
+        <v>29</v>
       </c>
       <c r="E5" t="s">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="F5" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="G5" t="s">
-        <v>59</v>
+        <v>42</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>52</v>
+        <v>37</v>
       </c>
       <c r="B6" t="s">
         <v>17</v>
       </c>
       <c r="C6" t="s">
-        <v>58</v>
+        <v>39</v>
       </c>
       <c r="D6" t="s">
-        <v>47</v>
+        <v>29</v>
       </c>
       <c r="E6" t="s">
+        <v>36</v>
+      </c>
+      <c r="F6" t="s">
         <v>24</v>
       </c>
-      <c r="F6" t="s">
-        <v>21</v>
-      </c>
       <c r="G6" t="s">
-        <v>60</v>
+        <v>43</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>52</v>
+        <v>37</v>
       </c>
       <c r="B7" t="s">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="C7" t="s">
-        <v>58</v>
+        <v>44</v>
       </c>
       <c r="D7" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="E7" t="s">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="F7" t="s">
-        <v>29</v>
+        <v>11</v>
       </c>
       <c r="G7" t="s">
-        <v>61</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>52</v>
+        <v>37</v>
       </c>
       <c r="B8" t="s">
+        <v>32</v>
+      </c>
+      <c r="C8" t="s">
+        <v>44</v>
+      </c>
+      <c r="D8" t="s">
+        <v>46</v>
+      </c>
+      <c r="E8" t="s">
         <v>31</v>
       </c>
-      <c r="C8" t="s">
-        <v>62</v>
-      </c>
-      <c r="D8" t="s">
-        <v>63</v>
-      </c>
-      <c r="E8" t="s">
-        <v>11</v>
-      </c>
       <c r="F8" t="s">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="G8" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>52</v>
-      </c>
-      <c r="B9" t="s">
-        <v>31</v>
-      </c>
-      <c r="C9" t="s">
-        <v>62</v>
-      </c>
-      <c r="D9" t="s">
-        <v>36</v>
-      </c>
-      <c r="E9" t="s">
-        <v>15</v>
-      </c>
-      <c r="F9" t="s">
-        <v>37</v>
-      </c>
-      <c r="G9" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -1158,7 +1076,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
@@ -1194,13 +1112,13 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>82</v>
       </c>
       <c r="B2" t="s">
         <v>8</v>
       </c>
       <c r="C2" t="s">
-        <v>9</v>
+        <v>83</v>
       </c>
       <c r="D2" t="s">
         <v>10</v>
@@ -1209,182 +1127,159 @@
         <v>11</v>
       </c>
       <c r="F2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="G2" t="s">
-        <v>13</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>82</v>
       </c>
       <c r="B3" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="C3" t="s">
-        <v>9</v>
+        <v>84</v>
       </c>
       <c r="D3" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="E3" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="F3" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="G3" t="s">
-        <v>13</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>82</v>
       </c>
       <c r="B4" t="s">
         <v>17</v>
       </c>
       <c r="C4" t="s">
-        <v>18</v>
+        <v>84</v>
       </c>
       <c r="D4" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="E4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F4" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="G4" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>7</v>
+        <v>82</v>
       </c>
       <c r="B5" t="s">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="C5" t="s">
-        <v>18</v>
+        <v>85</v>
       </c>
       <c r="D5" t="s">
-        <v>22</v>
+        <v>86</v>
       </c>
       <c r="E5" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="F5" t="s">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="G5" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>7</v>
+        <v>82</v>
       </c>
       <c r="B6" t="s">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="C6" t="s">
-        <v>18</v>
+        <v>85</v>
       </c>
       <c r="D6" t="s">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="E6" t="s">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="F6" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="G6" t="s">
-        <v>13</v>
+        <v>78</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>7</v>
+        <v>82</v>
       </c>
       <c r="B7" t="s">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="C7" t="s">
-        <v>18</v>
+        <v>85</v>
       </c>
       <c r="D7" t="s">
-        <v>28</v>
+        <v>55</v>
       </c>
       <c r="E7" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F7" t="s">
         <v>30</v>
       </c>
       <c r="G7" t="s">
-        <v>13</v>
+        <v>49</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>7</v>
+        <v>82</v>
       </c>
       <c r="B8" t="s">
-        <v>31</v>
+        <v>87</v>
       </c>
       <c r="C8" t="s">
-        <v>32</v>
+        <v>88</v>
       </c>
       <c r="D8" t="s">
-        <v>33</v>
+        <v>66</v>
       </c>
       <c r="E8" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F8" t="s">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="G8" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>7</v>
-      </c>
-      <c r="B9" t="s">
-        <v>31</v>
-      </c>
-      <c r="C9" t="s">
-        <v>32</v>
-      </c>
-      <c r="D9" t="s">
-        <v>36</v>
-      </c>
-      <c r="E9" t="s">
-        <v>37</v>
-      </c>
-      <c r="F9" t="s">
-        <v>38</v>
-      </c>
-      <c r="G9" t="s">
-        <v>13</v>
+        <v>56</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
@@ -1420,301 +1315,163 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>64</v>
+        <v>47</v>
       </c>
       <c r="B2" t="s">
-        <v>65</v>
+        <v>8</v>
       </c>
       <c r="C2" t="s">
-        <v>66</v>
+        <v>48</v>
       </c>
       <c r="D2" t="s">
-        <v>36</v>
+        <v>10</v>
       </c>
       <c r="E2" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="F2" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="G2" t="s">
-        <v>67</v>
+        <v>49</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>64</v>
+        <v>47</v>
       </c>
       <c r="B3" t="s">
-        <v>65</v>
+        <v>8</v>
       </c>
       <c r="C3" t="s">
-        <v>66</v>
+        <v>48</v>
       </c>
       <c r="D3" t="s">
-        <v>36</v>
+        <v>10</v>
       </c>
       <c r="E3" t="s">
-        <v>35</v>
+        <v>12</v>
       </c>
       <c r="F3" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="G3" t="s">
-        <v>55</v>
+        <v>42</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>64</v>
+        <v>47</v>
       </c>
       <c r="B4" t="s">
-        <v>65</v>
+        <v>17</v>
       </c>
       <c r="C4" t="s">
-        <v>66</v>
+        <v>50</v>
       </c>
       <c r="D4" t="s">
-        <v>41</v>
+        <v>51</v>
       </c>
       <c r="E4" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="F4" t="s">
-        <v>23</v>
+        <v>36</v>
       </c>
       <c r="G4" t="s">
-        <v>68</v>
+        <v>52</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>64</v>
+        <v>47</v>
       </c>
       <c r="B5" t="s">
-        <v>65</v>
+        <v>17</v>
       </c>
       <c r="C5" t="s">
-        <v>66</v>
+        <v>50</v>
       </c>
       <c r="D5" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="E5" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="F5" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="G5" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>64</v>
+        <v>47</v>
       </c>
       <c r="B6" t="s">
-        <v>65</v>
+        <v>17</v>
       </c>
       <c r="C6" t="s">
-        <v>66</v>
+        <v>50</v>
       </c>
       <c r="D6" t="s">
-        <v>56</v>
+        <v>29</v>
       </c>
       <c r="E6" t="s">
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="F6" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="G6" t="s">
-        <v>69</v>
+        <v>49</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>64</v>
+        <v>47</v>
       </c>
       <c r="B7" t="s">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="C7" t="s">
-        <v>70</v>
+        <v>54</v>
       </c>
       <c r="D7" t="s">
+        <v>55</v>
+      </c>
+      <c r="E7" t="s">
+        <v>15</v>
+      </c>
+      <c r="F7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G7" t="s">
         <v>56</v>
-      </c>
-      <c r="E7" t="s">
-        <v>29</v>
-      </c>
-      <c r="F7" t="s">
-        <v>12</v>
-      </c>
-      <c r="G7" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>64</v>
+        <v>47</v>
       </c>
       <c r="B8" t="s">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="C8" t="s">
-        <v>71</v>
+        <v>54</v>
       </c>
       <c r="D8" t="s">
-        <v>72</v>
+        <v>10</v>
       </c>
       <c r="E8" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="F8" t="s">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="G8" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>64</v>
-      </c>
-      <c r="B9" t="s">
-        <v>17</v>
-      </c>
-      <c r="C9" t="s">
-        <v>71</v>
-      </c>
-      <c r="D9" t="s">
-        <v>63</v>
-      </c>
-      <c r="E9" t="s">
-        <v>26</v>
-      </c>
-      <c r="F9" t="s">
-        <v>35</v>
-      </c>
-      <c r="G9" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>64</v>
-      </c>
-      <c r="B10" t="s">
-        <v>17</v>
-      </c>
-      <c r="C10" t="s">
-        <v>71</v>
-      </c>
-      <c r="D10" t="s">
-        <v>45</v>
-      </c>
-      <c r="E10" t="s">
-        <v>20</v>
-      </c>
-      <c r="F10" t="s">
-        <v>34</v>
-      </c>
-      <c r="G10" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>64</v>
-      </c>
-      <c r="B11" t="s">
-        <v>17</v>
-      </c>
-      <c r="C11" t="s">
-        <v>71</v>
-      </c>
-      <c r="D11" t="s">
-        <v>47</v>
-      </c>
-      <c r="E11" t="s">
-        <v>16</v>
-      </c>
-      <c r="F11" t="s">
-        <v>27</v>
-      </c>
-      <c r="G11" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>64</v>
-      </c>
-      <c r="B12" t="s">
-        <v>17</v>
-      </c>
-      <c r="C12" t="s">
-        <v>71</v>
-      </c>
-      <c r="D12" t="s">
-        <v>36</v>
-      </c>
-      <c r="E12" t="s">
-        <v>21</v>
-      </c>
-      <c r="F12" t="s">
-        <v>30</v>
-      </c>
-      <c r="G12" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>64</v>
-      </c>
-      <c r="B13" t="s">
-        <v>17</v>
-      </c>
-      <c r="C13" t="s">
-        <v>71</v>
-      </c>
-      <c r="D13" t="s">
-        <v>48</v>
-      </c>
-      <c r="E13" t="s">
-        <v>37</v>
-      </c>
-      <c r="F13" t="s">
-        <v>11</v>
-      </c>
-      <c r="G13" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>64</v>
-      </c>
-      <c r="B14" t="s">
-        <v>31</v>
-      </c>
-      <c r="C14" t="s">
-        <v>73</v>
-      </c>
-      <c r="D14" t="s">
-        <v>41</v>
-      </c>
-      <c r="E14" t="s">
-        <v>24</v>
-      </c>
-      <c r="F14" t="s">
-        <v>23</v>
-      </c>
-      <c r="G14" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>
@@ -1725,7 +1482,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
@@ -1761,186 +1518,163 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>74</v>
+        <v>57</v>
       </c>
       <c r="B2" t="s">
         <v>8</v>
       </c>
       <c r="C2" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="D2" t="s">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="E2" t="s">
-        <v>38</v>
+        <v>24</v>
       </c>
       <c r="F2" t="s">
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="G2" t="s">
-        <v>42</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>74</v>
+        <v>57</v>
       </c>
       <c r="B3" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="C3" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="D3" t="s">
-        <v>10</v>
+        <v>46</v>
       </c>
       <c r="E3" t="s">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="F3" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="G3" t="s">
-        <v>46</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>74</v>
+        <v>57</v>
       </c>
       <c r="B4" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="C4" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="D4" t="s">
-        <v>76</v>
+        <v>46</v>
       </c>
       <c r="E4" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" t="s">
         <v>12</v>
       </c>
-      <c r="F4" t="s">
-        <v>27</v>
-      </c>
       <c r="G4" t="s">
-        <v>77</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>74</v>
+        <v>57</v>
       </c>
       <c r="B5" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="C5" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="D5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E5" t="s">
+        <v>30</v>
+      </c>
+      <c r="F5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G5" t="s">
         <v>56</v>
-      </c>
-      <c r="E5" t="s">
-        <v>15</v>
-      </c>
-      <c r="F5" t="s">
-        <v>11</v>
-      </c>
-      <c r="G5" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>74</v>
+        <v>57</v>
       </c>
       <c r="B6" t="s">
         <v>17</v>
       </c>
       <c r="C6" t="s">
-        <v>79</v>
+        <v>59</v>
       </c>
       <c r="D6" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="E6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F6" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="G6" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>74</v>
+        <v>57</v>
       </c>
       <c r="B7" t="s">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="C7" t="s">
-        <v>79</v>
+        <v>61</v>
       </c>
       <c r="D7" t="s">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="E7" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="F7" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="G7" t="s">
-        <v>54</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>74</v>
+        <v>57</v>
       </c>
       <c r="B8" t="s">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="C8" t="s">
-        <v>79</v>
+        <v>61</v>
       </c>
       <c r="D8" t="s">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="E8" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="F8" t="s">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="G8" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>74</v>
-      </c>
-      <c r="B9" t="s">
-        <v>31</v>
-      </c>
-      <c r="C9" t="s">
-        <v>80</v>
-      </c>
-      <c r="D9" t="s">
-        <v>81</v>
-      </c>
-      <c r="E9" t="s">
-        <v>30</v>
-      </c>
-      <c r="F9" t="s">
-        <v>35</v>
-      </c>
-      <c r="G9" t="s">
-        <v>67</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -1951,7 +1685,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
@@ -1987,186 +1721,163 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>82</v>
+        <v>62</v>
       </c>
       <c r="B2" t="s">
         <v>8</v>
       </c>
       <c r="C2" t="s">
-        <v>83</v>
+        <v>63</v>
       </c>
       <c r="D2" t="s">
-        <v>47</v>
+        <v>64</v>
       </c>
       <c r="E2" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="F2" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="G2" t="s">
-        <v>84</v>
+        <v>65</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>82</v>
+        <v>62</v>
       </c>
       <c r="B3" t="s">
         <v>8</v>
       </c>
       <c r="C3" t="s">
-        <v>83</v>
+        <v>63</v>
       </c>
       <c r="D3" t="s">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="E3" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="F3" t="s">
-        <v>34</v>
+        <v>21</v>
       </c>
       <c r="G3" t="s">
-        <v>51</v>
+        <v>65</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>82</v>
+        <v>62</v>
       </c>
       <c r="B4" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="C4" t="s">
-        <v>85</v>
+        <v>63</v>
       </c>
       <c r="D4" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="E4" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
       <c r="F4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G4" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>82</v>
+        <v>62</v>
       </c>
       <c r="B5" t="s">
         <v>17</v>
       </c>
       <c r="C5" t="s">
-        <v>85</v>
+        <v>68</v>
       </c>
       <c r="D5" t="s">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="E5" t="s">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="F5" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="G5" t="s">
-        <v>57</v>
+        <v>69</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>82</v>
+        <v>62</v>
       </c>
       <c r="B6" t="s">
         <v>17</v>
       </c>
       <c r="C6" t="s">
-        <v>85</v>
+        <v>68</v>
       </c>
       <c r="D6" t="s">
-        <v>10</v>
+        <v>70</v>
       </c>
       <c r="E6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" t="s">
         <v>12</v>
       </c>
-      <c r="F6" t="s">
-        <v>21</v>
-      </c>
       <c r="G6" t="s">
-        <v>42</v>
+        <v>56</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>82</v>
+        <v>62</v>
       </c>
       <c r="B7" t="s">
         <v>17</v>
       </c>
       <c r="C7" t="s">
-        <v>85</v>
+        <v>68</v>
       </c>
       <c r="D7" t="s">
+        <v>40</v>
+      </c>
+      <c r="E7" t="s">
         <v>28</v>
       </c>
-      <c r="E7" t="s">
-        <v>26</v>
-      </c>
       <c r="F7" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="G7" t="s">
-        <v>86</v>
+        <v>56</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>82</v>
+        <v>62</v>
       </c>
       <c r="B8" t="s">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="C8" t="s">
-        <v>87</v>
+        <v>68</v>
       </c>
       <c r="D8" t="s">
-        <v>36</v>
+        <v>23</v>
       </c>
       <c r="E8" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="F8" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="G8" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>82</v>
-      </c>
-      <c r="B9" t="s">
-        <v>31</v>
-      </c>
-      <c r="C9" t="s">
-        <v>87</v>
-      </c>
-      <c r="D9" t="s">
-        <v>10</v>
-      </c>
-      <c r="E9" t="s">
-        <v>16</v>
-      </c>
-      <c r="F9" t="s">
-        <v>15</v>
-      </c>
-      <c r="G9" t="s">
-        <v>68</v>
+        <v>42</v>
       </c>
     </row>
   </sheetData>
@@ -2177,7 +1888,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
@@ -2213,186 +1924,163 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>88</v>
+        <v>71</v>
       </c>
       <c r="B2" t="s">
         <v>8</v>
       </c>
       <c r="C2" t="s">
-        <v>89</v>
+        <v>72</v>
       </c>
       <c r="D2" t="s">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="E2" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="F2" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="G2" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>88</v>
+        <v>71</v>
       </c>
       <c r="B3" t="s">
         <v>8</v>
       </c>
       <c r="C3" t="s">
-        <v>89</v>
+        <v>72</v>
       </c>
       <c r="D3" t="s">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="E3" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="F3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="G3" t="s">
-        <v>13</v>
+        <v>42</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>88</v>
+        <v>71</v>
       </c>
       <c r="B4" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="C4" t="s">
-        <v>89</v>
+        <v>73</v>
       </c>
       <c r="D4" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="E4" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="F4" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="G4" t="s">
-        <v>13</v>
+        <v>69</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>88</v>
+        <v>71</v>
       </c>
       <c r="B5" t="s">
         <v>17</v>
       </c>
       <c r="C5" t="s">
-        <v>90</v>
+        <v>73</v>
       </c>
       <c r="D5" t="s">
-        <v>72</v>
+        <v>23</v>
       </c>
       <c r="E5" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="F5" t="s">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="G5" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>88</v>
+        <v>71</v>
       </c>
       <c r="B6" t="s">
         <v>17</v>
       </c>
       <c r="C6" t="s">
-        <v>90</v>
+        <v>73</v>
       </c>
       <c r="D6" t="s">
-        <v>91</v>
+        <v>23</v>
       </c>
       <c r="E6" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="F6" t="s">
-        <v>92</v>
+        <v>11</v>
       </c>
       <c r="G6" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>88</v>
+        <v>71</v>
       </c>
       <c r="B7" t="s">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="C7" t="s">
-        <v>93</v>
+        <v>73</v>
       </c>
       <c r="D7" t="s">
-        <v>72</v>
+        <v>29</v>
       </c>
       <c r="E7" t="s">
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="F7" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G7" t="s">
-        <v>13</v>
+        <v>65</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>88</v>
+        <v>71</v>
       </c>
       <c r="B8" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C8" t="s">
-        <v>93</v>
+        <v>74</v>
       </c>
       <c r="D8" t="s">
-        <v>63</v>
+        <v>29</v>
       </c>
       <c r="E8" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F8" t="s">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="G8" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>88</v>
-      </c>
-      <c r="B9" t="s">
-        <v>31</v>
-      </c>
-      <c r="C9" t="s">
-        <v>93</v>
-      </c>
-      <c r="D9" t="s">
-        <v>45</v>
-      </c>
-      <c r="E9" t="s">
-        <v>29</v>
-      </c>
-      <c r="F9" t="s">
-        <v>27</v>
-      </c>
-      <c r="G9" t="s">
-        <v>13</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -2403,7 +2091,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
@@ -2439,190 +2127,167 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>94</v>
+        <v>75</v>
       </c>
       <c r="B2" t="s">
         <v>8</v>
       </c>
       <c r="C2" t="s">
-        <v>95</v>
+        <v>76</v>
       </c>
       <c r="D2" t="s">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="E2" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="F2" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="G2" t="s">
-        <v>13</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>94</v>
+        <v>75</v>
       </c>
       <c r="B3" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="C3" t="s">
-        <v>96</v>
+        <v>76</v>
       </c>
       <c r="D3" t="s">
-        <v>97</v>
+        <v>10</v>
       </c>
       <c r="E3" t="s">
         <v>27</v>
       </c>
       <c r="F3" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="G3" t="s">
-        <v>13</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>94</v>
+        <v>75</v>
       </c>
       <c r="B4" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="C4" t="s">
-        <v>96</v>
+        <v>76</v>
       </c>
       <c r="D4" t="s">
-        <v>98</v>
+        <v>66</v>
       </c>
       <c r="E4" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="F4" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="G4" t="s">
-        <v>13</v>
+        <v>42</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>94</v>
+        <v>75</v>
       </c>
       <c r="B5" t="s">
         <v>17</v>
       </c>
       <c r="C5" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="D5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E5" t="s">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="F5" t="s">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="G5" t="s">
-        <v>13</v>
+        <v>49</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>94</v>
+        <v>75</v>
       </c>
       <c r="B6" t="s">
         <v>17</v>
       </c>
       <c r="C6" t="s">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="D6" t="s">
-        <v>99</v>
+        <v>29</v>
       </c>
       <c r="E6" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="F6" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="G6" t="s">
-        <v>13</v>
+        <v>78</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>94</v>
+        <v>75</v>
       </c>
       <c r="B7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C7" t="s">
-        <v>100</v>
+        <v>79</v>
       </c>
       <c r="D7" t="s">
-        <v>97</v>
+        <v>80</v>
       </c>
       <c r="E7" t="s">
-        <v>35</v>
+        <v>12</v>
       </c>
       <c r="F7" t="s">
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="G7" t="s">
-        <v>13</v>
+        <v>52</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>94</v>
+        <v>75</v>
       </c>
       <c r="B8" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C8" t="s">
-        <v>100</v>
+        <v>79</v>
       </c>
       <c r="D8" t="s">
-        <v>63</v>
+        <v>81</v>
       </c>
       <c r="E8" t="s">
-        <v>92</v>
+        <v>14</v>
       </c>
       <c r="F8" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="G8" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>94</v>
-      </c>
-      <c r="B9" t="s">
-        <v>31</v>
-      </c>
-      <c r="C9" t="s">
-        <v>100</v>
-      </c>
-      <c r="D9" t="s">
-        <v>45</v>
-      </c>
-      <c r="E9" t="s">
         <v>26</v>
-      </c>
-      <c r="F9" t="s">
-        <v>38</v>
-      </c>
-      <c r="G9" t="s">
-        <v>13</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>